<commit_message>
Address review feedback: internal function, required column, simplified scenario logic
- Make .readIndividualParameterSetsFromXLS internal (no export)
- Remove species extraction; function now returns combined params structure
- Move per-sheet reading/combining logic into helper function
- Column 'Individual Parameter Sets' is now required in validation
- Remove species-specific param application from scenario.R
- Remove backward compatibility (no more sheet-named-after-individualId fallback)
- Add breaking change entry to NEWS.md
- Update vignettes/design-scenarios.Rmd
- Update tests: internal function via :::, validation tests include new column

Co-authored-by: PavelBal <25903040+PavelBal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/data/Individuals.xlsx
+++ b/tests/data/Individuals.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="IndividualBiometrics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ParamSet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -586,4 +587,60 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Container Path</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Parameter Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Organism|Kidney</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GFR</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ml/min</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>